<commit_message>
feat: add self-service change password endpoint for all users
</commit_message>
<xml_diff>
--- a/Teacher_Import_Template.xlsx
+++ b/Teacher_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6cddac052b6f52f/Desktop/School project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{074D331D-DB97-4261-BD94-A8BEA4FD99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{074D331D-DB97-4261-BD94-A8BEA4FD99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AD297B0-98D6-4C8C-B347-C2EDF4502D48}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{432B9544-194C-49B7-BA04-908ABA8B3323}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>serial_no</t>
   </si>
@@ -63,44 +63,20 @@
     <t>base_salary_per_day</t>
   </si>
   <si>
-    <t>Mrs. Priya Nair</t>
-  </si>
-  <si>
-    <t>priya.nair</t>
-  </si>
-  <si>
-    <t>Welcome@1</t>
-  </si>
-  <si>
     <t>TEACHER</t>
   </si>
   <si>
     <t>Class Teacher</t>
   </si>
   <si>
-    <t>Mr. Ramesh Verma</t>
-  </si>
-  <si>
-    <t>ramesh.verma</t>
-  </si>
-  <si>
-    <t>Subject Teacher</t>
-  </si>
-  <si>
-    <t>Dr. Anita Rao</t>
-  </si>
-  <si>
-    <t>anita.rao</t>
-  </si>
-  <si>
-    <t>Head of Department</t>
+    <t>Mrs. Chanda Kumari Yadav</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +88,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -140,14 +124,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -460,10 +447,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40F02D3-0294-4A19-AC43-F9BC07FB88FC}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="9" width="20.6328125" customWidth="1"/>
+    <col min="1" max="1" width="8.81640625" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
+    <col min="3" max="9" width="20.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -500,77 +489,17 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="H2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2">
-        <v>9876500001</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
       <c r="I2">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3">
-        <v>9876500002</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4">
-        <v>9876500003</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4">
-        <v>1000</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add clear-all-data endpoint and danger zone UI with double confirmation
</commit_message>
<xml_diff>
--- a/Teacher_Import_Template.xlsx
+++ b/Teacher_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f6cddac052b6f52f/Desktop/School project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{074D331D-DB97-4261-BD94-A8BEA4FD99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3AD297B0-98D6-4C8C-B347-C2EDF4502D48}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="8_{074D331D-DB97-4261-BD94-A8BEA4FD99F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D9303ED-1791-403C-B48E-6DAFDF1F8966}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{432B9544-194C-49B7-BA04-908ABA8B3323}"/>
   </bookViews>
@@ -69,7 +69,7 @@
     <t>Class Teacher</t>
   </si>
   <si>
-    <t>Mrs. Chanda Kumari Yadav</t>
+    <t>Chanda Kumari Yadav</t>
   </si>
 </sst>
 </file>
@@ -148,6 +148,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -495,6 +499,9 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
+      <c r="F2">
+        <v>7777777777</v>
+      </c>
       <c r="H2" t="s">
         <v>10</v>
       </c>

</xml_diff>